<commit_message>
Softball 2026-04-04: full pipeline run 2 (afternoon) — 7 stories, 5 articles, PostPlanner exports
New angles: A&M upsets No. 11 Georgia series win, Kendall Wells 29 HR NCAA freshman record chase,
FSU 23-game win streak, NCAA transfer portal window shift proposal, Red River Rivalry preview.
0 tweet char violations. Game 3 results (TX-AL/OU-KY) not indexed — covered forward-looking angles.
WordPress: blocked by proxy sandbox (known restriction).

https://claude.ai/code/session_0178Pb7ZnrqGqbWCLboPEiPL
</commit_message>
<xml_diff>
--- a/Softball/postplanner-imports/ils-postplanner-2026-04-04.xlsx
+++ b/Softball/postplanner-imports/ils-postplanner-2026-04-04.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/04/2026  17:15</t>
+          <t>04/04/2026  18:31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -492,7 +492,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/04/2026  17:30</t>
+          <t>04/04/2026  18:46</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/04/2026  17:45</t>
+          <t>04/04/2026  19:01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/04/2026  18:00</t>
+          <t>04/04/2026  19:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -535,7 +535,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/04/2026  18:15</t>
+          <t>04/04/2026  19:31</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -549,7 +549,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/04/2026  18:30</t>
+          <t>04/04/2026  19:46</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/04/2026  18:45</t>
+          <t>04/04/2026  20:01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -577,7 +577,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/04/2026  19:00</t>
+          <t>04/04/2026  20:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -592,7 +592,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04/04/2026  19:15</t>
+          <t>04/04/2026  20:31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -604,7 +604,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04/04/2026  19:30</t>
+          <t>04/04/2026  20:46</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -618,7 +618,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04/04/2026  19:45</t>
+          <t>04/04/2026  21:01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -633,7 +633,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04/04/2026  20:00</t>
+          <t>04/04/2026  21:16</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -649,7 +649,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04/04/2026  20:15</t>
+          <t>04/04/2026  21:31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04/04/2026  20:30</t>
+          <t>04/04/2026  21:46</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -676,7 +676,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04/04/2026  20:45</t>
+          <t>04/04/2026  22:01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04/04/2026  21:00</t>
+          <t>04/04/2026  22:16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -705,7 +705,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04/04/2026  21:15</t>
+          <t>04/04/2026  22:31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -720,7 +720,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04/04/2026  21:30</t>
+          <t>04/04/2026  22:46</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -736,7 +736,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04/04/2026  21:45</t>
+          <t>04/04/2026  23:01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -753,7 +753,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04/04/2026  22:00</t>
+          <t>04/04/2026  23:16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -765,7 +765,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04/04/2026  22:15</t>
+          <t>04/04/2026  23:31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04/04/2026  22:30</t>
+          <t>04/04/2026  23:46</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -800,7 +800,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04/04/2026  22:45</t>
+          <t>04/04/2026  23:45</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">

</xml_diff>